<commit_message>
Missing the 50000 line
</commit_message>
<xml_diff>
--- a/0.0 - Infrastructure around coding - VS Code/1.01 - Proposed Map.xlsx
+++ b/0.0 - Infrastructure around coding - VS Code/1.01 - Proposed Map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ellio\Documents\Python\A beginners guide to Python\0.0 - Infrastructure around coding - VS Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0EA71E6-6EE8-4D19-95F7-A60FC1237605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48AE0EB1-B3D0-4316-84B7-B67B51695617}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="21900" windowHeight="25296" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="3372" windowWidth="26004" windowHeight="21924" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="4.0 - Codeacademy" sheetId="4" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="142">
   <si>
     <t>Dipping the toe</t>
   </si>
@@ -443,6 +443,27 @@
   </si>
   <si>
     <t>Average</t>
+  </si>
+  <si>
+    <t>Out of place items</t>
+  </si>
+  <si>
+    <t>Key:</t>
+  </si>
+  <si>
+    <t>New subjects</t>
+  </si>
+  <si>
+    <t>Repeated subjects</t>
+  </si>
+  <si>
+    <t>Non-repeated subjects</t>
+  </si>
+  <si>
+    <t>Subjects covered twice</t>
+  </si>
+  <si>
+    <t>Covered but with a different name</t>
   </si>
 </sst>
 </file>
@@ -450,9 +471,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="177" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -507,8 +528,14 @@
       <name val="Aptos Light"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Light"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -533,8 +560,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF204056"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -601,11 +634,108 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -615,7 +745,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -630,15 +760,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -647,10 +788,10 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF204056"/>
+      <color rgb="FF8252DE"/>
       <color rgb="FFF20057"/>
       <color rgb="FFFFD636"/>
-      <color rgb="FF8252DE"/>
-      <color rgb="FF204056"/>
       <color rgb="FFFEF5F0"/>
       <color rgb="FFE7FFE7"/>
       <color rgb="FFFBFFFB"/>
@@ -2180,16 +2321,57 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15B86D8A-CBC0-49C9-9806-C0813A4AC871}">
-  <dimension ref="A4:M78"/>
+  <dimension ref="A1:M79"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="20.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="24.88671875" customWidth="1"/>
+    <col min="5" max="5" width="24.88671875" customWidth="1"/>
+    <col min="6" max="6" width="30.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9" customWidth="1"/>
     <col min="10" max="10" width="36.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="52.5546875" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" s="2"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+    </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
@@ -2198,6 +2380,10 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
@@ -2205,8 +2391,14 @@
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
+      <c r="F5" s="24" t="s">
+        <v>136</v>
+      </c>
       <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
     </row>
     <row r="6" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2"/>
@@ -2217,9 +2409,15 @@
       <c r="D6" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="2"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="31" t="s">
+        <v>135</v>
+      </c>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="23"/>
+      <c r="K6" s="2"/>
     </row>
     <row r="7" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
@@ -2229,8 +2427,12 @@
         <v>2</v>
       </c>
       <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
+      <c r="F7" s="25"/>
       <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
       <c r="M7" t="s">
         <v>33</v>
       </c>
@@ -2239,12 +2441,16 @@
       <c r="A8" s="2"/>
       <c r="B8" s="3"/>
       <c r="C8" s="4"/>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="21" t="s">
         <v>3</v>
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
     </row>
     <row r="9" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2"/>
@@ -2256,6 +2462,10 @@
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
       <c r="M9" t="s">
         <v>34</v>
       </c>
@@ -2268,6 +2478,10 @@
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
     </row>
     <row r="11" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2"/>
@@ -2277,6 +2491,10 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
       <c r="M11" t="s">
         <v>35</v>
       </c>
@@ -2295,6 +2513,10 @@
         <v>7</v>
       </c>
       <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="2"/>
       <c r="M12" t="s">
         <v>36</v>
       </c>
@@ -2307,6 +2529,10 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
     </row>
     <row r="14" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
@@ -2320,6 +2546,10 @@
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
       <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
       <c r="M14" t="s">
         <v>37</v>
       </c>
@@ -2334,6 +2564,10 @@
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
       <c r="M15" t="s">
         <v>38</v>
       </c>
@@ -2348,6 +2582,10 @@
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
       <c r="M16" t="s">
         <v>39</v>
       </c>
@@ -2362,17 +2600,25 @@
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
     </row>
     <row r="18" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="21" t="s">
         <v>8</v>
       </c>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
       <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
       <c r="M18" t="s">
         <v>40</v>
       </c>
@@ -2387,6 +2633,10 @@
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
       <c r="M19" t="s">
         <v>41</v>
       </c>
@@ -2399,10 +2649,14 @@
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="21" t="s">
         <v>27</v>
       </c>
       <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
       <c r="M20" t="s">
         <v>42</v>
       </c>
@@ -2417,17 +2671,25 @@
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
     </row>
     <row r="22" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2"/>
       <c r="B22" s="3"/>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="21" t="s">
         <v>15</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
       <c r="M22" t="s">
         <v>43</v>
       </c>
@@ -2442,6 +2704,10 @@
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
       <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
       <c r="M23" t="s">
         <v>44</v>
       </c>
@@ -2456,6 +2722,10 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
     </row>
     <row r="25" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
@@ -2467,6 +2737,10 @@
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
       <c r="M25" t="s">
         <v>45</v>
       </c>
@@ -2483,6 +2757,10 @@
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
       <c r="M26" t="s">
         <v>46</v>
       </c>
@@ -2497,6 +2775,10 @@
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
     </row>
     <row r="28" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
@@ -2506,6 +2788,10 @@
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
       <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
       <c r="M28" t="s">
         <v>47</v>
       </c>
@@ -2520,6 +2806,10 @@
         <v>25</v>
       </c>
       <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
+      <c r="K29" s="2"/>
       <c r="M29" t="s">
         <v>48</v>
       </c>
@@ -2534,6 +2824,10 @@
         <v>28</v>
       </c>
       <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2"/>
+      <c r="K30" s="2"/>
     </row>
     <row r="31" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
@@ -2545,6 +2839,10 @@
         <v>26</v>
       </c>
       <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
       <c r="M31" t="s">
         <v>49</v>
       </c>
@@ -2559,6 +2857,10 @@
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
       <c r="M32" t="s">
         <v>50</v>
       </c>
@@ -2568,11 +2870,15 @@
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
-      <c r="E33" s="4" t="s">
+      <c r="E33" s="21" t="s">
         <v>22</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2"/>
+      <c r="K33" s="2"/>
       <c r="M33" t="s">
         <v>51</v>
       </c>
@@ -2587,6 +2893,10 @@
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
     </row>
     <row r="35" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
@@ -2598,6 +2908,10 @@
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
+      <c r="K35" s="2"/>
       <c r="M35" t="s">
         <v>52</v>
       </c>
@@ -2612,6 +2926,10 @@
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
       <c r="M36" t="s">
         <v>53</v>
       </c>
@@ -2624,6 +2942,10 @@
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="2"/>
+      <c r="K37" s="2"/>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
@@ -2633,18 +2955,51 @@
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="4"/>
+      <c r="K38" s="2"/>
       <c r="M38" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="4"/>
+      <c r="K39" s="2"/>
       <c r="M39" t="s">
         <v>55</v>
       </c>
     </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+      <c r="J40" s="4"/>
+      <c r="K40" s="2"/>
+    </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
+      <c r="K41" s="2"/>
       <c r="M41" t="s">
         <v>56</v>
       </c>
@@ -2659,6 +3014,7 @@
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
+      <c r="K42" s="2"/>
       <c r="M42" t="s">
         <v>57</v>
       </c>
@@ -2668,11 +3024,14 @@
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
-      <c r="F43" s="2"/>
+      <c r="F43" s="24" t="s">
+        <v>136</v>
+      </c>
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
+      <c r="K43" s="2"/>
     </row>
     <row r="44" spans="1:13" ht="18" x14ac:dyDescent="0.35">
       <c r="B44" s="3" t="s">
@@ -2682,14 +3041,17 @@
       <c r="D44" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="E44" s="4"/>
-      <c r="F44" s="4"/>
-      <c r="G44" s="2"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="G44" s="23"/>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
       <c r="J44" s="4" t="s">
         <v>79</v>
       </c>
+      <c r="K44" s="2"/>
       <c r="M44" t="s">
         <v>58</v>
       </c>
@@ -2700,13 +3062,17 @@
       <c r="D45" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E45" s="4"/>
-      <c r="G45" s="2"/>
+      <c r="E45" s="22"/>
+      <c r="F45" s="27" t="s">
+        <v>139</v>
+      </c>
+      <c r="G45" s="23"/>
       <c r="H45" s="2"/>
       <c r="I45" s="2"/>
       <c r="J45" s="4" t="s">
         <v>80</v>
       </c>
+      <c r="K45" s="2"/>
       <c r="M45" t="s">
         <v>59</v>
       </c>
@@ -2717,14 +3083,17 @@
       <c r="D46" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="2"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="28" t="s">
+        <v>137</v>
+      </c>
+      <c r="G46" s="23"/>
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
       <c r="J46" s="4" t="s">
         <v>124</v>
       </c>
+      <c r="K46" s="2"/>
     </row>
     <row r="47" spans="1:13" ht="18" x14ac:dyDescent="0.35">
       <c r="B47" s="3"/>
@@ -2732,13 +3101,16 @@
       <c r="D47" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="F47" s="4"/>
-      <c r="G47" s="2"/>
+      <c r="F47" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="G47" s="23"/>
       <c r="H47" s="2"/>
       <c r="I47" s="2"/>
       <c r="J47" s="4" t="s">
         <v>81</v>
       </c>
+      <c r="K47" s="2"/>
       <c r="M47" t="s">
         <v>60</v>
       </c>
@@ -2747,14 +3119,17 @@
       <c r="B48" s="3"/>
       <c r="C48" s="4"/>
       <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4"/>
-      <c r="G48" s="2"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="30" t="s">
+        <v>141</v>
+      </c>
+      <c r="G48" s="23"/>
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
       <c r="J48" s="4" t="s">
         <v>125</v>
       </c>
+      <c r="K48" s="2"/>
       <c r="M48" t="s">
         <v>61</v>
       </c>
@@ -2763,356 +3138,374 @@
       <c r="B49" s="3"/>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4"/>
-      <c r="G49" s="2"/>
+      <c r="E49" s="22"/>
+      <c r="F49" s="25"/>
+      <c r="G49" s="23"/>
       <c r="H49" s="2"/>
       <c r="I49" s="2"/>
-      <c r="J49" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="J49" s="4"/>
+      <c r="K49" s="2"/>
     </row>
     <row r="50" spans="2:13" ht="18" x14ac:dyDescent="0.35">
       <c r="B50" s="3"/>
       <c r="C50" s="4"/>
-      <c r="D50" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E50" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F50" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G50" s="5"/>
-      <c r="H50" s="5"/>
-      <c r="I50" s="5"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="25"/>
+      <c r="G50" s="2"/>
+      <c r="H50" s="2"/>
+      <c r="I50" s="2"/>
       <c r="J50" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="M50" t="s">
-        <v>62</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="K50" s="2"/>
     </row>
     <row r="51" spans="2:13" ht="18" x14ac:dyDescent="0.35">
       <c r="B51" s="3"/>
       <c r="C51" s="4"/>
-      <c r="D51" s="4"/>
-      <c r="E51" s="4"/>
-      <c r="F51" s="4"/>
-      <c r="G51" s="2"/>
-      <c r="H51" s="2"/>
-      <c r="I51" s="2"/>
+      <c r="D51" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5"/>
+      <c r="I51" s="5"/>
       <c r="J51" s="4" t="s">
-        <v>83</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="K51" s="2"/>
       <c r="M51" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="52" spans="2:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B52" s="3" t="s">
-        <v>5</v>
-      </c>
+      <c r="B52" s="3"/>
       <c r="C52" s="4"/>
-      <c r="D52" s="7" t="s">
-        <v>109</v>
-      </c>
+      <c r="D52" s="4"/>
       <c r="E52" s="4"/>
-      <c r="F52" s="8" t="s">
-        <v>91</v>
-      </c>
+      <c r="F52" s="4"/>
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>
       <c r="I52" s="2"/>
       <c r="J52" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
+      </c>
+      <c r="K52" s="2"/>
+      <c r="M52" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="53" spans="2:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B53" s="3"/>
+      <c r="B53" s="3" t="s">
+        <v>5</v>
+      </c>
       <c r="C53" s="4"/>
       <c r="D53" s="7" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="E53" s="4"/>
-      <c r="F53" s="4"/>
+      <c r="F53" s="8" t="s">
+        <v>91</v>
+      </c>
       <c r="G53" s="2"/>
       <c r="H53" s="2"/>
       <c r="I53" s="2"/>
       <c r="J53" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="M53" t="s">
-        <v>64</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="K53" s="2"/>
     </row>
     <row r="54" spans="2:13" ht="18" x14ac:dyDescent="0.35">
       <c r="B54" s="3"/>
       <c r="C54" s="4"/>
-      <c r="D54" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="E54" s="7" t="s">
-        <v>93</v>
-      </c>
+      <c r="D54" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="E54" s="4"/>
       <c r="F54" s="4"/>
       <c r="G54" s="2"/>
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
       <c r="J54" s="4" t="s">
-        <v>86</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="K54" s="2"/>
       <c r="M54" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="55" spans="2:13" ht="18" x14ac:dyDescent="0.35">
       <c r="B55" s="3"/>
       <c r="C55" s="4"/>
+      <c r="D55" s="4" t="s">
+        <v>94</v>
+      </c>
       <c r="E55" s="7" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F55" s="4"/>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
       <c r="I55" s="2"/>
       <c r="J55" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="56" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B56" s="4"/>
+        <v>86</v>
+      </c>
+      <c r="K55" s="2"/>
+      <c r="M55" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="56" spans="2:13" ht="18" x14ac:dyDescent="0.35">
+      <c r="B56" s="3"/>
       <c r="C56" s="4"/>
-      <c r="D56" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="E56" s="4" t="s">
-        <v>101</v>
+      <c r="E56" s="7" t="s">
+        <v>97</v>
       </c>
       <c r="F56" s="4"/>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>
       <c r="J56" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="M56" t="s">
-        <v>66</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="K56" s="2"/>
     </row>
     <row r="57" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="E57" s="4"/>
-      <c r="F57" s="8" t="s">
-        <v>105</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="F57" s="4"/>
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
       <c r="J57" s="4" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="58" spans="2:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B58" s="3"/>
+        <v>127</v>
+      </c>
+      <c r="K57" s="2"/>
+      <c r="M57" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="58" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B58" s="4"/>
       <c r="C58" s="4"/>
-      <c r="D58" s="7" t="s">
-        <v>96</v>
+      <c r="D58" s="4" t="s">
+        <v>99</v>
       </c>
       <c r="E58" s="4"/>
-      <c r="F58" s="4"/>
+      <c r="F58" s="8" t="s">
+        <v>105</v>
+      </c>
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>
       <c r="J58" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="M58" t="s">
-        <v>67</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="K58" s="2"/>
     </row>
     <row r="59" spans="2:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B59" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="B59" s="3"/>
       <c r="C59" s="4"/>
       <c r="D59" s="7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E59" s="4"/>
-      <c r="F59" s="10" t="s">
-        <v>27</v>
-      </c>
+      <c r="F59" s="4"/>
       <c r="G59" s="2"/>
       <c r="H59" s="2"/>
       <c r="I59" s="2"/>
       <c r="J59" s="4" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="60" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B60" s="4"/>
+        <v>129</v>
+      </c>
+      <c r="K59" s="2"/>
+      <c r="M59" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="60" spans="2:13" ht="18" x14ac:dyDescent="0.35">
+      <c r="B60" s="6" t="s">
+        <v>13</v>
+      </c>
       <c r="C60" s="4"/>
-      <c r="D60" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="E60" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="F60" s="4"/>
+      <c r="D60" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E60" s="4"/>
+      <c r="F60" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
       <c r="I60" s="2"/>
       <c r="J60" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="M60" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="61" spans="2:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B61" s="3"/>
+        <v>130</v>
+      </c>
+      <c r="K60" s="2"/>
+    </row>
+    <row r="61" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B61" s="4"/>
       <c r="C61" s="4"/>
-      <c r="D61" s="4"/>
-      <c r="E61" s="4" t="s">
-        <v>102</v>
+      <c r="D61" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E61" s="7" t="s">
+        <v>95</v>
       </c>
       <c r="F61" s="4"/>
       <c r="G61" s="2"/>
       <c r="H61" s="2"/>
       <c r="I61" s="2"/>
       <c r="J61" s="4" t="s">
-        <v>132</v>
-      </c>
+        <v>131</v>
+      </c>
+      <c r="K61" s="2"/>
       <c r="M61" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="62" spans="2:13" ht="18" x14ac:dyDescent="0.35">
       <c r="B62" s="3"/>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
-      <c r="E62" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F62" s="9"/>
+      <c r="E62" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F62" s="4"/>
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
       <c r="J62" s="4" t="s">
-        <v>88</v>
+        <v>132</v>
+      </c>
+      <c r="K62" s="2"/>
+      <c r="M62" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="63" spans="2:13" ht="18" x14ac:dyDescent="0.35">
       <c r="B63" s="3"/>
       <c r="C63" s="4"/>
-      <c r="D63" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E63" s="2"/>
-      <c r="F63" s="2"/>
+      <c r="D63" s="4"/>
+      <c r="E63" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F63" s="9"/>
       <c r="G63" s="2"/>
       <c r="H63" s="2"/>
       <c r="I63" s="2"/>
       <c r="J63" s="4" t="s">
-        <v>89</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="K63" s="2"/>
     </row>
     <row r="64" spans="2:13" ht="18" x14ac:dyDescent="0.35">
       <c r="B64" s="3"/>
       <c r="C64" s="4"/>
-      <c r="D64" s="4"/>
+      <c r="D64" s="10" t="s">
+        <v>9</v>
+      </c>
       <c r="E64" s="2"/>
       <c r="F64" s="2"/>
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
       <c r="J64" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="K64" s="2"/>
+    </row>
+    <row r="65" spans="2:13" ht="18" x14ac:dyDescent="0.35">
+      <c r="B65" s="3"/>
+      <c r="C65" s="4"/>
+      <c r="D65" s="4"/>
+      <c r="E65" s="2"/>
+      <c r="F65" s="2"/>
+      <c r="G65" s="2"/>
+      <c r="H65" s="2"/>
+      <c r="I65" s="2"/>
+      <c r="J65" s="4" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="65" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B65" s="4"/>
-      <c r="C65" s="4"/>
-      <c r="D65" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="E65" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="F65" s="4"/>
-      <c r="G65" s="2"/>
-      <c r="I65" s="2"/>
-      <c r="M65" t="s">
-        <v>70</v>
-      </c>
+      <c r="K65" s="2"/>
     </row>
     <row r="66" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
-      <c r="D66" s="4" t="s">
-        <v>104</v>
+      <c r="D66" s="10" t="s">
+        <v>23</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F66" s="4"/>
       <c r="G66" s="2"/>
-      <c r="H66" s="2"/>
       <c r="I66" s="2"/>
-      <c r="J66" s="2"/>
+      <c r="K66" s="2"/>
       <c r="M66" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="67" spans="2:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B67" s="3" t="s">
-        <v>18</v>
-      </c>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="67" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B67" s="4"/>
       <c r="C67" s="4"/>
-      <c r="D67" s="4"/>
-      <c r="E67" s="10" t="s">
-        <v>21</v>
+      <c r="D67" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E67" s="4" t="s">
+        <v>106</v>
       </c>
       <c r="F67" s="4"/>
       <c r="G67" s="2"/>
       <c r="H67" s="2"/>
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
-    </row>
-    <row r="68" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B68" s="4"/>
+      <c r="K67" s="2"/>
+      <c r="M67" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="68" spans="2:13" ht="18" x14ac:dyDescent="0.35">
+      <c r="B68" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
       <c r="E68" s="10" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F68" s="4"/>
       <c r="G68" s="2"/>
       <c r="H68" s="2"/>
       <c r="I68" s="2"/>
       <c r="J68" s="2"/>
-      <c r="M68" t="s">
-        <v>72</v>
-      </c>
+      <c r="K68" s="2"/>
     </row>
     <row r="69" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
-      <c r="E69" s="4"/>
+      <c r="E69" s="10" t="s">
+        <v>30</v>
+      </c>
       <c r="F69" s="4"/>
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
+      <c r="K69" s="2"/>
       <c r="M69" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="70" spans="2:13" x14ac:dyDescent="0.3">
@@ -3120,13 +3513,15 @@
       <c r="C70" s="4"/>
       <c r="D70" s="4"/>
       <c r="E70" s="4"/>
-      <c r="F70" s="10" t="s">
-        <v>25</v>
-      </c>
+      <c r="F70" s="4"/>
       <c r="G70" s="2"/>
       <c r="H70" s="2"/>
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
+      <c r="K70" s="2"/>
+      <c r="M70" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="71" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B71" s="4"/>
@@ -3134,116 +3529,138 @@
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
       <c r="F71" s="10" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G71" s="2"/>
       <c r="H71" s="2"/>
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
-      <c r="M71" t="s">
-        <v>74</v>
-      </c>
+      <c r="K71" s="2"/>
     </row>
     <row r="72" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B72" s="4"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
-      <c r="F72" s="7" t="s">
-        <v>108</v>
+      <c r="F72" s="10" t="s">
+        <v>28</v>
       </c>
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
+      <c r="K72" s="2"/>
       <c r="M72" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="73" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B73" s="4"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
-      <c r="E73" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="F73" s="4"/>
+      <c r="E73" s="4"/>
+      <c r="F73" s="7" t="s">
+        <v>108</v>
+      </c>
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
+      <c r="K73" s="2"/>
+      <c r="M73" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="74" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B74" s="4"/>
       <c r="C74" s="4"/>
       <c r="D74" s="4"/>
       <c r="E74" s="10" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="F74" s="4"/>
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
-      <c r="M74" t="s">
-        <v>76</v>
-      </c>
+      <c r="K74" s="2"/>
     </row>
     <row r="75" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B75" s="4"/>
       <c r="C75" s="4"/>
       <c r="D75" s="4"/>
-      <c r="E75" s="11" t="s">
-        <v>24</v>
+      <c r="E75" s="10" t="s">
+        <v>22</v>
       </c>
       <c r="F75" s="4"/>
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
       <c r="I75" s="2"/>
       <c r="J75" s="2"/>
+      <c r="K75" s="2"/>
       <c r="M75" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="76" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B76" s="4"/>
       <c r="C76" s="4"/>
       <c r="D76" s="4"/>
-      <c r="E76" s="10" t="s">
-        <v>29</v>
+      <c r="E76" s="11" t="s">
+        <v>24</v>
       </c>
       <c r="F76" s="4"/>
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
+      <c r="K76" s="2"/>
+      <c r="M76" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="77" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B77" s="4"/>
       <c r="C77" s="4"/>
       <c r="D77" s="4"/>
       <c r="E77" s="10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F77" s="4"/>
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
-      <c r="M77" t="s">
-        <v>78</v>
-      </c>
+      <c r="K77" s="2"/>
     </row>
     <row r="78" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B78" s="4"/>
       <c r="C78" s="4"/>
       <c r="D78" s="4"/>
-      <c r="E78" s="4"/>
+      <c r="E78" s="10" t="s">
+        <v>31</v>
+      </c>
       <c r="F78" s="4"/>
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
       <c r="I78" s="2"/>
       <c r="J78" s="2"/>
+      <c r="K78" s="2"/>
+      <c r="M78" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="79" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B79" s="4"/>
+      <c r="C79" s="4"/>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4"/>
+      <c r="F79" s="4"/>
+      <c r="G79" s="2"/>
+      <c r="H79" s="2"/>
+      <c r="I79" s="2"/>
+      <c r="J79" s="2"/>
+      <c r="K79" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>